<commit_message>
metamaterials fig3 script updates
</commit_message>
<xml_diff>
--- a/Ricochet/helper_codes/Ricochet Collaboration Membership.xlsx
+++ b/Ricochet/helper_codes/Ricochet Collaboration Membership.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiatongy/Project_codes/Jiatong-Yang/Ricochet/helper_codes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE2866B3-545C-1F46-B927-95AD8ABE34A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB565423-3CD1-ED40-B55C-34C5FA755B8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Membership" sheetId="2" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="651" uniqueCount="306">
   <si>
     <t>Institution</t>
   </si>
@@ -2912,7 +2912,9 @@
       <c r="E83" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="F83" s="5"/>
+      <c r="F83" s="5" t="s">
+        <v>304</v>
+      </c>
       <c r="G83" s="5"/>
       <c r="H83" s="5"/>
       <c r="I83" s="5"/>
@@ -3111,6 +3113,9 @@
       <c r="E92" s="4" t="s">
         <v>28</v>
       </c>
+      <c r="F92" s="2" t="s">
+        <v>304</v>
+      </c>
     </row>
     <row r="93" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="5" t="s">
@@ -3144,6 +3149,9 @@
       </c>
       <c r="E94" s="4" t="s">
         <v>28</v>
+      </c>
+      <c r="F94" s="2" t="s">
+        <v>304</v>
       </c>
     </row>
     <row r="95" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3747,6 +3755,9 @@
       </c>
       <c r="E127" s="6" t="s">
         <v>28</v>
+      </c>
+      <c r="F127" s="11" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="128" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4689,7 +4700,7 @@
     <row r="1042" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <phoneticPr fontId="9" type="noConversion"/>
-  <conditionalFormatting sqref="E1:F26 A1:D80 F27:F38 E39:F46 E67:F72 E74:F74 B81:D82 A81:A112 E83:F83 A83:D94 F84 E85:F87 F92:F112 B95:D112 F113:K115 A113:E128 B129:E129 A130:E1042 G1 F116:F126 F129:F1042 F47:F82 E89:F91 E27:E112">
+  <conditionalFormatting sqref="G1 E1:F26 A1:D80 F27:F38 E27:E112 E39:F46 F47:F82 E67:F72 E74:F74 B81:D82 A81:A112 E83:F83 A83:D94 F84 E85:F87 E89:F91 F92:F112 B95:D112 F113:K115 A113:E128 F116:F126 B129:E129 F129:F1042 A130:E1042">
     <cfRule type="expression" dxfId="0" priority="5">
       <formula>#REF!="No"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Updated uMUX paper editing stuff
</commit_message>
<xml_diff>
--- a/Ricochet/helper_codes/Ricochet Collaboration Membership.xlsx
+++ b/Ricochet/helper_codes/Ricochet Collaboration Membership.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiatongy/Project_codes/Jiatong-Yang/Ricochet/helper_codes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB565423-3CD1-ED40-B55C-34C5FA755B8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6275AA01-90BE-EB42-8476-9C5EBE5D7CBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Membership" sheetId="2" r:id="rId1"/>
@@ -866,9 +866,6 @@
     <t>Caitlyn</t>
   </si>
   <si>
-    <t>Department of Physics, University of Toronto, ON, Canada</t>
-  </si>
-  <si>
     <t xml:space="preserve">Univ Lyon, Université Lyon 1, CNRS/IN2P3, IP2I-Lyon, F-69622, Villeurbanne, France </t>
   </si>
   <si>
@@ -951,6 +948,9 @@
   </si>
   <si>
     <t>Research Laboratory of Electronics, Massachusetts Institute of Technology, Cambridge, MA, USA 02139</t>
+  </si>
+  <si>
+    <t>Department of Physics, University of Toronto, ON, Canada M5S 1A7</t>
   </si>
 </sst>
 </file>
@@ -1321,15 +1321,15 @@
         <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>302</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>303</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>5</v>
@@ -1346,7 +1346,7 @@
     </row>
     <row r="3" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>8</v>
@@ -1363,7 +1363,7 @@
     </row>
     <row r="4" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>11</v>
@@ -1380,7 +1380,7 @@
     </row>
     <row r="5" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>14</v>
@@ -1403,7 +1403,7 @@
     </row>
     <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>17</v>
@@ -1426,7 +1426,7 @@
     </row>
     <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>19</v>
@@ -1449,7 +1449,7 @@
     </row>
     <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>21</v>
@@ -1472,7 +1472,7 @@
     </row>
     <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>24</v>
@@ -1495,7 +1495,7 @@
     </row>
     <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>27</v>
@@ -1518,7 +1518,7 @@
     </row>
     <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>29</v>
@@ -1541,7 +1541,7 @@
     </row>
     <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>32</v>
@@ -1564,7 +1564,7 @@
     </row>
     <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>33</v>
@@ -1587,7 +1587,7 @@
     </row>
     <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>36</v>
@@ -1610,7 +1610,7 @@
     </row>
     <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>39</v>
@@ -1633,7 +1633,7 @@
     </row>
     <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>42</v>
@@ -1651,7 +1651,7 @@
     </row>
     <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>45</v>
@@ -1669,7 +1669,7 @@
     </row>
     <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>48</v>
@@ -1686,7 +1686,7 @@
     </row>
     <row r="19" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>51</v>
@@ -1703,7 +1703,7 @@
     </row>
     <row r="20" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B20" s="7" t="s">
         <v>53</v>
@@ -1721,7 +1721,7 @@
     </row>
     <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B21" s="7" t="s">
         <v>55</v>
@@ -1738,7 +1738,7 @@
     </row>
     <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B22" s="7" t="s">
         <v>57</v>
@@ -1755,7 +1755,7 @@
     </row>
     <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B23" s="7" t="s">
         <v>60</v>
@@ -1772,7 +1772,7 @@
     </row>
     <row r="24" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B24" s="7" t="s">
         <v>63</v>
@@ -1789,7 +1789,7 @@
     </row>
     <row r="25" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B25" s="7" t="s">
         <v>65</v>
@@ -1806,7 +1806,7 @@
     </row>
     <row r="26" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B26" s="7" t="s">
         <v>68</v>
@@ -1823,7 +1823,7 @@
     </row>
     <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>71</v>
@@ -1840,7 +1840,7 @@
     </row>
     <row r="28" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>73</v>
@@ -1857,7 +1857,7 @@
     </row>
     <row r="29" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>75</v>
@@ -1874,7 +1874,7 @@
     </row>
     <row r="30" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>77</v>
@@ -1892,7 +1892,7 @@
     </row>
     <row r="31" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>79</v>
@@ -1909,7 +1909,7 @@
     </row>
     <row r="32" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>82</v>
@@ -1926,7 +1926,7 @@
     </row>
     <row r="33" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>84</v>
@@ -1943,7 +1943,7 @@
     </row>
     <row r="34" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>85</v>
@@ -1960,7 +1960,7 @@
     </row>
     <row r="35" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>87</v>
@@ -1977,7 +1977,7 @@
     </row>
     <row r="36" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>89</v>
@@ -1994,7 +1994,7 @@
     </row>
     <row r="37" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B37" s="6" t="s">
         <v>91</v>
@@ -2012,7 +2012,7 @@
     </row>
     <row r="38" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>93</v>
@@ -2029,7 +2029,7 @@
     </row>
     <row r="39" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>96</v>
@@ -2052,7 +2052,7 @@
     </row>
     <row r="40" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>98</v>
@@ -2075,7 +2075,7 @@
     </row>
     <row r="41" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>100</v>
@@ -2098,7 +2098,7 @@
     </row>
     <row r="42" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>102</v>
@@ -2121,7 +2121,7 @@
     </row>
     <row r="43" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>106</v>
@@ -2144,7 +2144,7 @@
     </row>
     <row r="44" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>107</v>
@@ -2167,7 +2167,7 @@
     </row>
     <row r="45" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>108</v>
@@ -2190,7 +2190,7 @@
     </row>
     <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>111</v>
@@ -2213,7 +2213,7 @@
     </row>
     <row r="47" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>113</v>
@@ -2230,7 +2230,7 @@
     </row>
     <row r="48" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>114</v>
@@ -2247,7 +2247,7 @@
     </row>
     <row r="49" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>116</v>
@@ -2264,7 +2264,7 @@
     </row>
     <row r="50" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>118</v>
@@ -2282,7 +2282,7 @@
     </row>
     <row r="51" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>119</v>
@@ -2299,7 +2299,7 @@
     </row>
     <row r="52" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>121</v>
@@ -2316,7 +2316,7 @@
     </row>
     <row r="53" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>122</v>
@@ -2334,7 +2334,7 @@
     </row>
     <row r="54" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>124</v>
@@ -2351,7 +2351,7 @@
     </row>
     <row r="55" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>126</v>
@@ -2368,7 +2368,7 @@
     </row>
     <row r="56" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>129</v>
@@ -2386,7 +2386,7 @@
     </row>
     <row r="57" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>131</v>
@@ -2403,7 +2403,7 @@
     </row>
     <row r="58" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>133</v>
@@ -2420,7 +2420,7 @@
     </row>
     <row r="59" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>135</v>
@@ -2437,7 +2437,7 @@
     </row>
     <row r="60" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>137</v>
@@ -2455,7 +2455,7 @@
     </row>
     <row r="61" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B61" s="2" t="s">
         <v>139</v>
@@ -2472,7 +2472,7 @@
     </row>
     <row r="62" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>141</v>
@@ -2489,7 +2489,7 @@
     </row>
     <row r="63" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>144</v>
@@ -2507,7 +2507,7 @@
     </row>
     <row r="64" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B64" s="2" t="s">
         <v>146</v>
@@ -2525,7 +2525,7 @@
     </row>
     <row r="65" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B65" s="2" t="s">
         <v>148</v>
@@ -2543,7 +2543,7 @@
     </row>
     <row r="66" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B66" s="9" t="s">
         <v>148</v>
@@ -2704,7 +2704,7 @@
     </row>
     <row r="73" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B73" s="2" t="s">
         <v>166</v>
@@ -2721,7 +2721,7 @@
     </row>
     <row r="74" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>168</v>
@@ -2744,7 +2744,7 @@
     </row>
     <row r="75" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B75" s="2" t="s">
         <v>170</v>
@@ -2762,7 +2762,7 @@
     </row>
     <row r="76" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B76" s="2" t="s">
         <v>172</v>
@@ -2780,7 +2780,7 @@
     </row>
     <row r="77" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B77" s="2" t="s">
         <v>133</v>
@@ -2798,7 +2798,7 @@
     </row>
     <row r="78" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B78" s="6" t="s">
         <v>174</v>
@@ -2815,7 +2815,7 @@
     </row>
     <row r="79" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B79" s="6" t="s">
         <v>176</v>
@@ -2832,7 +2832,7 @@
     </row>
     <row r="80" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B80" s="6" t="s">
         <v>178</v>
@@ -2850,7 +2850,7 @@
     </row>
     <row r="81" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B81" s="2" t="s">
         <v>180</v>
@@ -2873,7 +2873,7 @@
     </row>
     <row r="82" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>182</v>
@@ -2888,7 +2888,7 @@
         <v>28</v>
       </c>
       <c r="F82" s="6" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="G82" s="5"/>
       <c r="H82" s="5"/>
@@ -2898,7 +2898,7 @@
     </row>
     <row r="83" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B83" s="2" t="s">
         <v>185</v>
@@ -2913,7 +2913,7 @@
         <v>28</v>
       </c>
       <c r="F83" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="G83" s="5"/>
       <c r="H83" s="5"/>
@@ -2923,7 +2923,7 @@
     </row>
     <row r="84" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B84" s="2" t="s">
         <v>187</v>
@@ -2941,7 +2941,7 @@
     </row>
     <row r="85" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B85" s="2" t="s">
         <v>190</v>
@@ -2964,7 +2964,7 @@
     </row>
     <row r="86" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B86" s="2" t="s">
         <v>193</v>
@@ -2987,7 +2987,7 @@
     </row>
     <row r="87" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B87" s="2" t="s">
         <v>195</v>
@@ -3010,7 +3010,7 @@
     </row>
     <row r="88" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B88" s="2" t="s">
         <v>197</v>
@@ -3025,12 +3025,12 @@
         <v>28</v>
       </c>
       <c r="F88" s="11" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="89" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B89" s="2" t="s">
         <v>200</v>
@@ -3053,7 +3053,7 @@
     </row>
     <row r="90" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B90" s="2" t="s">
         <v>202</v>
@@ -3076,7 +3076,7 @@
     </row>
     <row r="91" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B91" s="2" t="s">
         <v>204</v>
@@ -3099,7 +3099,7 @@
     </row>
     <row r="92" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B92" s="9" t="s">
         <v>207</v>
@@ -3114,12 +3114,12 @@
         <v>28</v>
       </c>
       <c r="F92" s="2" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="93" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B93" s="9" t="s">
         <v>210</v>
@@ -3136,7 +3136,7 @@
     </row>
     <row r="94" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B94" s="9" t="s">
         <v>212</v>
@@ -3151,12 +3151,12 @@
         <v>28</v>
       </c>
       <c r="F94" s="2" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="95" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B95" s="2" t="s">
         <v>214</v>
@@ -3179,7 +3179,7 @@
     </row>
     <row r="96" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B96" s="2" t="s">
         <v>217</v>
@@ -3197,7 +3197,7 @@
     </row>
     <row r="97" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B97" s="2" t="s">
         <v>220</v>
@@ -3214,7 +3214,7 @@
     </row>
     <row r="98" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B98" s="2" t="s">
         <v>222</v>
@@ -3301,7 +3301,7 @@
     </row>
     <row r="103" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="6" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B103" s="2" t="s">
         <v>231</v>
@@ -3319,7 +3319,7 @@
     </row>
     <row r="104" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="6" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B104" s="9" t="s">
         <v>233</v>
@@ -3336,7 +3336,7 @@
     </row>
     <row r="105" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="6" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B105" s="9" t="s">
         <v>235</v>
@@ -3353,7 +3353,7 @@
     </row>
     <row r="106" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="6" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B106" s="9" t="s">
         <v>237</v>
@@ -3370,7 +3370,7 @@
     </row>
     <row r="107" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="6" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B107" s="9" t="s">
         <v>239</v>
@@ -3387,7 +3387,7 @@
     </row>
     <row r="108" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="6" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B108" s="9" t="s">
         <v>241</v>
@@ -3404,7 +3404,7 @@
     </row>
     <row r="109" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="6" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B109" s="9" t="s">
         <v>243</v>
@@ -3421,7 +3421,7 @@
     </row>
     <row r="110" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="6" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B110" s="9" t="s">
         <v>246</v>
@@ -3438,7 +3438,7 @@
     </row>
     <row r="111" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="6" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B111" s="9" t="s">
         <v>247</v>
@@ -3455,7 +3455,7 @@
     </row>
     <row r="112" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="6" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B112" s="9" t="s">
         <v>249</v>
@@ -3472,7 +3472,7 @@
     </row>
     <row r="113" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="2" t="s">
-        <v>277</v>
+        <v>305</v>
       </c>
       <c r="B113" s="2" t="s">
         <v>259</v>
@@ -3495,7 +3495,7 @@
     </row>
     <row r="114" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="2" t="s">
-        <v>277</v>
+        <v>305</v>
       </c>
       <c r="B114" s="2" t="s">
         <v>262</v>
@@ -3518,7 +3518,7 @@
     </row>
     <row r="115" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="2" t="s">
-        <v>277</v>
+        <v>305</v>
       </c>
       <c r="B115" s="2" t="s">
         <v>264</v>
@@ -3541,7 +3541,7 @@
     </row>
     <row r="116" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B116" s="2" t="s">
         <v>266</v>
@@ -3558,7 +3558,7 @@
     </row>
     <row r="117" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B117" s="9" t="s">
         <v>269</v>
@@ -3581,7 +3581,7 @@
     </row>
     <row r="118" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B118" s="6" t="s">
         <v>271</v>
@@ -3598,7 +3598,7 @@
     </row>
     <row r="119" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B119" s="6" t="s">
         <v>273</v>
@@ -3615,7 +3615,7 @@
     </row>
     <row r="120" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B120" s="6" t="s">
         <v>275</v>
@@ -3632,7 +3632,7 @@
     </row>
     <row r="121" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="11" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B121" s="9" t="s">
         <v>251</v>
@@ -3647,15 +3647,15 @@
         <v>28</v>
       </c>
       <c r="F121" s="6" t="s">
+        <v>303</v>
+      </c>
+      <c r="G121" s="11" t="s">
         <v>304</v>
-      </c>
-      <c r="G121" s="11" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="122" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" s="11" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B122" s="9" t="s">
         <v>254</v>
@@ -3673,7 +3673,7 @@
     </row>
     <row r="123" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="11" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B123" s="9" t="s">
         <v>257</v>
@@ -3691,16 +3691,16 @@
     </row>
     <row r="124" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="11" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B124" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="C124" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="C124" s="2" t="s">
+      <c r="D124" s="2" t="s">
         <v>288</v>
-      </c>
-      <c r="D124" s="2" t="s">
-        <v>289</v>
       </c>
       <c r="E124" s="6" t="s">
         <v>28</v>
@@ -3708,16 +3708,16 @@
     </row>
     <row r="125" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="11" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C125" s="2" t="s">
         <v>267</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E125" s="6" t="s">
         <v>28</v>
@@ -3725,16 +3725,16 @@
     </row>
     <row r="126" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="11" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B126" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="C126" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="C126" s="2" t="s">
+      <c r="D126" s="2" t="s">
         <v>293</v>
-      </c>
-      <c r="D126" s="2" t="s">
-        <v>294</v>
       </c>
       <c r="E126" s="6" t="s">
         <v>28</v>
@@ -3742,42 +3742,42 @@
     </row>
     <row r="127" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="11" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B127" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="C127" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="C127" s="2" t="s">
-        <v>297</v>
-      </c>
       <c r="D127" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E127" s="6" t="s">
         <v>28</v>
       </c>
       <c r="F127" s="11" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="128" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B128" s="2" t="s">
         <v>193</v>
       </c>
       <c r="C128" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="D128" s="2" t="s">
         <v>300</v>
       </c>
-      <c r="D128" s="2" t="s">
-        <v>301</v>
-      </c>
       <c r="E128" s="6" t="s">
         <v>28</v>
       </c>
       <c r="F128" s="11" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="129" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>